<commit_message>
Clean directory structure, add sidebar auth, and display academic metrics chart
</commit_message>
<xml_diff>
--- a/ecv_data.xlsx
+++ b/ecv_data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\alip2\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\alip2\cv_portfolio\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6B3D72E-71E7-42C4-AA84-3A2450807723}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7200286-A5C9-456E-ADC4-8B20079904D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Profil" sheetId="1" r:id="rId1"/>
@@ -18,13 +18,14 @@
     <sheet name="Projects" sheetId="3" r:id="rId3"/>
     <sheet name="Activities" sheetId="4" r:id="rId4"/>
     <sheet name="Certifications" sheetId="5" r:id="rId5"/>
+    <sheet name="Academic_data" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="126">
   <si>
     <t>Field</t>
   </si>
@@ -384,6 +385,24 @@
   </si>
   <si>
     <t>https://drive.google.com/file/d/1lL-lD2DbWn6SlqRAzZmD0tmuISuoOH4_/view?usp=sharing</t>
+  </si>
+  <si>
+    <t>Semester</t>
+  </si>
+  <si>
+    <t>IPK</t>
+  </si>
+  <si>
+    <t>Link_Bukti</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/19AVhYXw4JYyko9K3et49Uc9sGhkI4YPr/view?usp=sharing</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1TlKqckdJRgjOSX-qKfQ0XwZtqhgxWwYr/view?usp=sharing</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1nXY17I6CrErAyPQm_NEax_75C9rTV8uJ/view?usp=sharing</t>
   </si>
 </sst>
 </file>
@@ -911,7 +930,7 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="42"/>
     <xf numFmtId="0" fontId="19" fillId="33" borderId="10" xfId="42" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -923,6 +942,7 @@
     <xf numFmtId="0" fontId="20" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1872,4 +1892,66 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DFFF97C1-60D2-4E8E-A3D7-0A9897A8169E}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="6.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>120</v>
+      </c>
+      <c r="B1" t="s">
+        <v>121</v>
+      </c>
+      <c r="C1" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="5">
+        <v>4</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" s="5">
+        <v>4</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>3.87</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C2" r:id="rId1" xr:uid="{5908AFBF-6BE0-4FC0-806D-F5A2980888E6}"/>
+    <hyperlink ref="C3" r:id="rId2" xr:uid="{97C3BE15-A6C5-4002-974C-020B05AF529E}"/>
+    <hyperlink ref="C4" r:id="rId3" xr:uid="{7828DDD8-08C2-473E-BB4C-D3460922EFB1}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>